<commit_message>
Review EFSA PEC soil degradation parameters
- The pseudo-DT50 values calculated from FOMC/3.32 or log(2)/k2 are now
  more accurately called substitute half-lives in the comments and the
  derappp vignette.
- Substitute half-lives are given to a maximum of four significant digits
- A large substitute half-life was added for fluxapyroxad, while a
  substitute half-life derived from the worst-case lab soil was not
  entered for dimethomorph, as it seems too high given the field
  dissipation data available
- For spirotetramat, EFSA used the worst-case lab value of 0.33 days
  instead of the worst-case non-normalised field DT50 of 1 day.
  Elisabeth had proposed to use 1 day, as we use worst-case
  non-normalised field in most cases. I propose to accept this with
  a comment, as I do not consider field dissipation data wrong just
  because they show slower degradation than in the lab.
- For cymoxanil, I added the latest value from the 2026 EFSA conclusion.
</commit_message>
<xml_diff>
--- a/data_generation/07_soil_degradation/soil_degradation_EFSA_PEC_soil_roan_luel_first_ai.xlsx
+++ b/data_generation/07_soil_degradation/soil_degradation_EFSA_PEC_soil_roan_luel_first_ai.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\07_soil_degradation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A742276-AEF7-48D1-B481-A12A97BB8A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{921D5CB7-594A-445D-96E6-D548AC5E8934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24105" yWindow="195" windowWidth="19185" windowHeight="11265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle2" sheetId="2" r:id="rId1"/>
-    <sheet name="Tabelle3" sheetId="3" r:id="rId2"/>
+    <sheet name="Soil degradation" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle2!$A$1:$Q$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Soil degradation'!$A$1:$Q$61</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="174">
   <si>
     <t>Amisulbrom</t>
   </si>
@@ -49,18 +48,12 @@
     <t>SFO</t>
   </si>
   <si>
-    <t>EFSA Journal 2014;12(4):3237</t>
-  </si>
-  <si>
     <t>Azoxystrobin</t>
   </si>
   <si>
     <t>Benalaxyl</t>
   </si>
   <si>
-    <t>EFSA Journal 2020;18(1):5985</t>
-  </si>
-  <si>
     <t>Bixafen</t>
   </si>
   <si>
@@ -97,21 +90,12 @@
     <t>Cyproconazole</t>
   </si>
   <si>
-    <t>EFSA Journal 2010;8(11):1897</t>
-  </si>
-  <si>
     <t>Cyprodinil</t>
   </si>
   <si>
-    <t>EFSA Journal 2025:9209</t>
-  </si>
-  <si>
     <t>Difenoconazole</t>
   </si>
   <si>
-    <t>EFSA Journal 2011;9(1):1967</t>
-  </si>
-  <si>
     <t>Diflufenican</t>
   </si>
   <si>
@@ -133,9 +117,6 @@
     <t>Fenpyroximate</t>
   </si>
   <si>
-    <t>EFSA Journal 2013;11(12):3493</t>
-  </si>
-  <si>
     <t>Fludioxonil</t>
   </si>
   <si>
@@ -166,24 +147,15 @@
     <t>Linuron</t>
   </si>
   <si>
-    <t>EFSA Journal 2016;14(7):4518</t>
-  </si>
-  <si>
     <t>Mandipropamid</t>
   </si>
   <si>
     <t xml:space="preserve">SFO </t>
   </si>
   <si>
-    <t>EFSA Journal 2012;10(11):2935</t>
-  </si>
-  <si>
     <t>Mepanipyrim</t>
   </si>
   <si>
-    <t>EFSA Journal 2017;15(6):4852</t>
-  </si>
-  <si>
     <t>Metamitron</t>
   </si>
   <si>
@@ -205,15 +177,9 @@
     <t>Pendimethalin</t>
   </si>
   <si>
-    <t>EFSA Journal 2016;14(3):4420</t>
-  </si>
-  <si>
     <t>Pethoxamid</t>
   </si>
   <si>
-    <t>EFSA Journal 2017;15(9):4981</t>
-  </si>
-  <si>
     <t>Picoxystrobin</t>
   </si>
   <si>
@@ -238,21 +204,12 @@
     <t>S-Metolachlor</t>
   </si>
   <si>
-    <t>EFSA Journal 2023:7852</t>
-  </si>
-  <si>
     <t>Tebuconazole</t>
   </si>
   <si>
-    <t>EFSA Journal 2014;12(1):3485</t>
-  </si>
-  <si>
     <t>Tebufenozide</t>
   </si>
   <si>
-    <t>EFSA Journal 2010;8(12):1871</t>
-  </si>
-  <si>
     <t>Tebufenpyrad</t>
   </si>
   <si>
@@ -262,15 +219,9 @@
     <t>Thiacloprid</t>
   </si>
   <si>
-    <t>EFSA Journal 2019;17(3):559</t>
-  </si>
-  <si>
     <t>Trifloxystrobin</t>
   </si>
   <si>
-    <t>EFSA Journal 2017;15(10):4989</t>
-  </si>
-  <si>
     <t>substance</t>
   </si>
   <si>
@@ -370,48 +321,21 @@
     <t>j.efsa.2013.3493</t>
   </si>
   <si>
-    <t>j.efsa.2019.559</t>
-  </si>
-  <si>
     <t>j.efsa.2017.4981</t>
   </si>
   <si>
-    <t>j.efsa.2023.8373</t>
-  </si>
-  <si>
-    <t>EFSA Journal 2009;7(10):1350</t>
-  </si>
-  <si>
     <t>j.efsa.2009.1350</t>
   </si>
   <si>
-    <t>EFSA Journal 2010;8(4):1542</t>
-  </si>
-  <si>
     <t>j.efsa.2010.1542</t>
   </si>
   <si>
-    <t>EFSA Journal 2010;8(4):1565</t>
-  </si>
-  <si>
     <t>j.efsa.2010.1565</t>
   </si>
   <si>
-    <t>EFSA Journal 2010;8(5):1598</t>
-  </si>
-  <si>
     <t>j.efsa.2010.1598</t>
   </si>
   <si>
-    <t>EFSA Journal 2010;8(6):162</t>
-  </si>
-  <si>
-    <t>j.efsa.2010.162</t>
-  </si>
-  <si>
-    <t>EFSA Journal 2010;8(9):1707</t>
-  </si>
-  <si>
     <t>j.efsa.2010.1707</t>
   </si>
   <si>
@@ -421,12 +345,6 @@
     <t>j.efsa.2010.1871</t>
   </si>
   <si>
-    <t>EFSA Journal 2011;9(1):196</t>
-  </si>
-  <si>
-    <t>j.efsa.2011.196</t>
-  </si>
-  <si>
     <t>j.efsa.2011.1967</t>
   </si>
   <si>
@@ -436,9 +354,6 @@
     <t>j.efsa.2014.3485</t>
   </si>
   <si>
-    <t>EFSA Journal 2016;14(1):4374</t>
-  </si>
-  <si>
     <t>j.efsa.2016.4374</t>
   </si>
   <si>
@@ -457,12 +372,6 @@
     <t>j.efsa.2023.7852</t>
   </si>
   <si>
-    <t>EFSA Journal 2023:8373</t>
-  </si>
-  <si>
-    <t>EFSA Journal 2024:8997</t>
-  </si>
-  <si>
     <t>j.efsa.2024.8997</t>
   </si>
   <si>
@@ -499,36 +408,15 @@
     <t>j.efsa.2009.299r</t>
   </si>
   <si>
-    <t>DT50 37 recorded on page 39 for PEC soil calculation is not a half life</t>
-  </si>
-  <si>
-    <t>calculated from DT90 396 [d]/3.32</t>
-  </si>
-  <si>
-    <t>DT50 50.6 recorded for PEC soil calculation is not a half life, as in pseudo DT50 calculated from DT90!</t>
-  </si>
-  <si>
-    <t>DT50 1235 recorded on page 42 for PEC soil calculation is not a half life, as in pseudo DT50 calculated from LN(2)/k2!!</t>
-  </si>
-  <si>
     <t>k1 and k2 calculated from  1.DT50 = 20.327 days; 2.DT50 = 495.105 days</t>
   </si>
   <si>
-    <t>calculated from DT90 515/3.32 on page 34</t>
-  </si>
-  <si>
     <t>DT50</t>
   </si>
   <si>
     <t>kinetics</t>
   </si>
   <si>
-    <t>Pseudo-SFO (backcalculated from FOMC DT90 7544.7 days/3.32)</t>
-  </si>
-  <si>
-    <t>Pseudo-SFO (ln(2)/k2)</t>
-  </si>
-  <si>
     <t>FALSE</t>
   </si>
   <si>
@@ -574,9 +462,6 @@
     <t>j.efsa.2025.9206</t>
   </si>
   <si>
-    <t>DT50 calculated from ln(2)/k2</t>
-  </si>
-  <si>
     <t>j.efsa.2024.9047</t>
   </si>
   <si>
@@ -625,9 +510,6 @@
     <t>EU Review report</t>
   </si>
   <si>
-    <t>worst case field DT50</t>
-  </si>
-  <si>
     <t>outdated via 2024 EFSA Conclusion</t>
   </si>
   <si>
@@ -649,7 +531,37 @@
     <t>Used for Southern Europe by EFSA</t>
   </si>
   <si>
-    <t xml:space="preserve">370 DT50 on page 49 is not a pseudo DT50 calculated from DT90 &gt;1000/3.32 </t>
+    <t>DT50 50.6 recorded for PEC soil calculation is not a half life substitute, so we calculated one from the FOMC DT90 divided by 3.32</t>
+  </si>
+  <si>
+    <t>Substitute half-life calculated from ln(2)/k2</t>
+  </si>
+  <si>
+    <t>Substitute half-life calculated from DT90 396 [d]/3.32</t>
+  </si>
+  <si>
+    <t>Substitute half-life calculated from DT90 515 on page 34 divided by 3.32</t>
+  </si>
+  <si>
+    <t>370 d DT50 on page 49 is not a substitute half-life but the time for reaching 50% the first time for the FOMC fit to the Wilson, UK field study. We calculated a substitute half-life from the FOMC parameters as DT90/3.32</t>
+  </si>
+  <si>
+    <t>roan, luel</t>
+  </si>
+  <si>
+    <t>roan, luel, rajo</t>
+  </si>
+  <si>
+    <t>DT50 37 recorded on page 39 for PEC soil calculation is not a substitute half life, so we give a substitute half-life from the worst-case field DT90 (FOMC) divided by 3.32 (p. 30)</t>
+  </si>
+  <si>
+    <t>DT50 1235 recorded on page 42 for PEC soil calculation is not a substitute half-life, so we backcalculated one from ln(2)/k2</t>
+  </si>
+  <si>
+    <t>Substitute half-life (ln(2)/k2)</t>
+  </si>
+  <si>
+    <t>Substitute half-life (backcalculated from FOMC DT90 7544.7 days/3.32)</t>
   </si>
 </sst>
 </file>
@@ -697,24 +609,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -729,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -740,13 +640,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1028,83 +928,84 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44ABC253-0668-4FE2-BC14-84FC263B038A}">
   <dimension ref="A1:R61"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.54296875" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" customWidth="1"/>
-    <col min="4" max="4" width="9.90625" customWidth="1"/>
-    <col min="5" max="6" width="5.90625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.08984375" style="3" customWidth="1"/>
-    <col min="8" max="8" width="9.54296875" style="3" customWidth="1"/>
-    <col min="9" max="10" width="5.90625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="6" width="11.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" style="3" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="8.08984375" customWidth="1"/>
-    <col min="13" max="13" width="10.08984375" customWidth="1"/>
-    <col min="14" max="14" width="19.26953125" customWidth="1"/>
-    <col min="15" max="15" width="35.90625" customWidth="1"/>
-    <col min="16" max="16" width="9.54296875" customWidth="1"/>
+    <col min="12" max="12" width="8.140625" customWidth="1"/>
+    <col min="13" max="13" width="10.140625" customWidth="1"/>
+    <col min="14" max="14" width="15.5703125" customWidth="1"/>
+    <col min="15" max="15" width="35.85546875" customWidth="1"/>
+    <col min="16" max="16" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>147</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>158</v>
+        <v>123</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>159</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C2" s="4">
         <v>12.6</v>
@@ -1112,38 +1013,31 @@
       <c r="D2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
       <c r="K2" s="4" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="L2" s="4">
         <v>42</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O2" s="4"/>
+        <v>76</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>77</v>
+      </c>
       <c r="P2" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C3" s="4">
         <v>262</v>
@@ -1152,30 +1046,31 @@
         <v>1</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="L3" s="4">
         <v>40</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>93</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="O3" s="10"/>
       <c r="P3" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C4" s="4">
         <v>127.6</v>
@@ -1184,116 +1079,115 @@
         <v>1</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>136</v>
+        <v>108</v>
       </c>
       <c r="L4" s="4">
         <v>43</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="4">
+        <v>3014</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <v>8.0999999999999996E-3</v>
+      </c>
+      <c r="H5" s="4">
+        <v>2.3000000000000001E-4</v>
+      </c>
+      <c r="J5" s="4">
+        <v>53</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="L5" s="4">
+        <v>42</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C5" s="6">
-        <f>LN(2)/H5</f>
-        <v>3013.6833937388924</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="4">
+        <v>227.4</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="L6" s="4">
+        <v>59</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6">
-        <v>8.0999999999999996E-3</v>
-      </c>
-      <c r="H5" s="6">
-        <v>2.3000000000000001E-4</v>
-      </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6">
-        <v>53</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="L5" s="6">
-        <v>42</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q5" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" s="4">
+        <v>119.3</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C6" s="6">
-        <v>227.4</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="L6" s="6">
-        <v>59</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="P6" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C7" s="4">
-        <v>119.277</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>10</v>
       </c>
       <c r="E7" s="4">
         <v>1.1222700000000001</v>
@@ -1302,33 +1196,33 @@
         <v>58.398800000000001</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="L7" s="5">
         <v>39</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O7" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q7" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="P7" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C8" s="4">
         <v>166.2</v>
@@ -1337,30 +1231,30 @@
         <v>1</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>167</v>
+        <v>130</v>
       </c>
       <c r="L8" s="4">
         <v>54</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C9" s="4">
         <v>78</v>
@@ -1369,30 +1263,30 @@
         <v>1</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="L9" s="4">
         <v>32</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C10" s="4">
         <v>78.5</v>
@@ -1401,30 +1295,30 @@
         <v>1</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="L10" s="4">
         <v>55</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>187</v>
+        <v>149</v>
       </c>
       <c r="C11" s="4">
         <v>107.2</v>
@@ -1433,30 +1327,30 @@
         <v>1</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>175</v>
+        <v>138</v>
       </c>
       <c r="L11" s="4">
         <v>43</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>188</v>
+        <v>150</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q11" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>187</v>
+        <v>149</v>
       </c>
       <c r="C12" s="4">
         <v>88.9</v>
@@ -1465,30 +1359,30 @@
         <v>1</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>173</v>
+        <v>136</v>
       </c>
       <c r="L12" s="4">
         <v>64</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>188</v>
+        <v>150</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C13" s="4">
         <v>90</v>
@@ -1497,30 +1391,30 @@
         <v>1</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="L13" s="4">
         <v>46</v>
       </c>
-      <c r="M13" s="9" t="s">
-        <v>162</v>
+      <c r="M13" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>189</v>
+        <v>151</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q13" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C14" s="4">
         <v>195</v>
@@ -1529,27 +1423,30 @@
         <v>1</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>176</v>
+        <v>139</v>
       </c>
       <c r="L14" s="4">
         <v>39</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C15" s="4">
         <v>141.30000000000001</v>
@@ -1558,30 +1455,30 @@
         <v>1</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="L15" s="4">
         <v>40</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C16" s="4">
         <v>284.3</v>
@@ -1590,30 +1487,30 @@
         <v>1</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="L16" s="4">
         <v>41</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C17" s="4">
         <v>265</v>
@@ -1622,30 +1519,30 @@
         <v>1</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="L17" s="4">
         <v>39</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C18" s="4">
         <v>645</v>
@@ -1654,30 +1551,30 @@
         <v>1</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>190</v>
+        <v>152</v>
       </c>
       <c r="L18" s="4">
         <v>68</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C19" s="4">
         <v>231</v>
@@ -1686,30 +1583,30 @@
         <v>1</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="L19" s="4">
         <v>46</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C20" s="4">
         <v>226</v>
@@ -1718,30 +1615,30 @@
         <v>1</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="L20" s="4">
         <v>61</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P20" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q20" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C21" s="4">
         <v>157</v>
@@ -1750,30 +1647,30 @@
         <v>1</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="L21" s="4">
         <v>72</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P21" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q21" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C22" s="4">
         <v>116</v>
@@ -1781,81 +1678,72 @@
       <c r="D22" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
       <c r="K22" s="4" t="s">
-        <v>169</v>
+        <v>132</v>
       </c>
       <c r="L22" s="4">
         <v>57</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="N22" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O22" s="4"/>
+        <v>76</v>
+      </c>
+      <c r="N22" s="4" t="s">
+        <v>77</v>
+      </c>
       <c r="P22" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q22" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
-        <v>28</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C23" s="6">
-        <v>1350.6020000000001</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E23" s="6">
+        <v>148</v>
+      </c>
+      <c r="C23" s="4">
+        <v>1351</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="4">
         <v>0.37330000000000002</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="4">
         <v>9.4143000000000008</v>
       </c>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="L23" s="6">
+      <c r="K23" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="L23" s="4">
         <v>62</v>
       </c>
-      <c r="M23" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="N23" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O23" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="P23" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q23" s="6"/>
-    </row>
-    <row r="24" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M23" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="N23" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q23" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C24" s="3">
         <v>16.7</v>
@@ -1864,31 +1752,31 @@
         <v>1</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="L24" s="4">
         <v>47</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O24" s="3"/>
       <c r="P24" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C25" s="3">
         <v>43</v>
@@ -1897,37 +1785,36 @@
         <v>1</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="L25" s="4">
         <v>56</v>
       </c>
-      <c r="M25" s="10" t="s">
-        <v>162</v>
+      <c r="M25" s="8" t="s">
+        <v>125</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>195</v>
+        <v>156</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q25" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C26" s="3">
-        <f>LN(2)/H26</f>
-        <v>1848.3924814931875</v>
+        <v>1848</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G26" s="3">
         <v>0.01</v>
@@ -1939,33 +1826,33 @@
         <v>22.08</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="L26" s="4">
         <v>39</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="Q26" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C27" s="3">
         <v>68.099999999999994</v>
@@ -1974,31 +1861,31 @@
         <v>1</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="L27" s="4">
         <v>70</v>
       </c>
       <c r="M27" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O27" s="3"/>
       <c r="P27" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q27" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C28" s="3">
         <v>290</v>
@@ -2013,37 +1900,37 @@
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="L28" s="3">
         <v>99</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O28" s="3"/>
       <c r="P28" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C29" s="4">
-        <v>495.10500000000002</v>
+        <v>495.1</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
@@ -2060,33 +1947,33 @@
       </c>
       <c r="J29" s="4"/>
       <c r="K29" s="4" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="L29" s="4">
         <v>39</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>156</v>
+        <v>122</v>
       </c>
       <c r="P29" s="4" t="s">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="Q29" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="3" t="s">
-        <v>36</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C30" s="3">
         <v>119</v>
@@ -2101,37 +1988,37 @@
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>171</v>
+        <v>134</v>
       </c>
       <c r="L30" s="3">
         <v>61</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O30" s="3"/>
       <c r="P30" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C31" s="4">
-        <v>154.96</v>
+        <v>155</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E31" s="4">
         <v>1.1299999999999999</v>
@@ -2144,116 +2031,109 @@
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="L31" s="7">
+        <v>87</v>
+      </c>
+      <c r="L31" s="6">
         <v>36</v>
       </c>
       <c r="M31" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q31" s="4"/>
-    </row>
-    <row r="32" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="C32" s="3">
+        <v>79</v>
+      </c>
+      <c r="Q31" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C32" s="4">
         <v>240</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="L32" s="3">
+      <c r="D32" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="L32" s="4">
         <v>12</v>
       </c>
-      <c r="M32" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="N32" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="O32" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="P32" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q32" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C33" s="6">
-        <f>1000/3.32</f>
-        <v>301.20481927710847</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="6">
+      <c r="M32" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="N32" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="P32" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q32" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C33" s="3">
+        <v>284400</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="3">
         <v>0.2059</v>
       </c>
-      <c r="F33" s="6">
+      <c r="F33" s="3">
         <v>13.1342</v>
       </c>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="L33" s="6">
+      <c r="K33" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L33" s="3">
         <v>49</v>
       </c>
-      <c r="M33" s="6" t="s">
-        <v>92</v>
+      <c r="M33" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O33" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="P33" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q33" s="6"/>
-    </row>
-    <row r="34" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+      <c r="O33" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="P33" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q33" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C34" s="3">
         <v>168.4</v>
@@ -2262,63 +2142,63 @@
         <v>1</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="L34" s="3">
         <v>29</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O34" s="3"/>
       <c r="P34" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C35" s="3">
         <v>72.3</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>129</v>
+        <v>102</v>
       </c>
       <c r="L35" s="3">
         <v>43</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C36" s="3">
         <v>82.1</v>
@@ -2327,31 +2207,31 @@
         <v>1</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
       <c r="L36" s="3">
         <v>47</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O36" s="3"/>
       <c r="P36" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>163</v>
+        <v>126</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C37" s="3">
         <v>30.9</v>
@@ -2360,33 +2240,33 @@
         <v>1</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>165</v>
+        <v>128</v>
       </c>
       <c r="L37" s="3">
         <v>20</v>
       </c>
       <c r="M37" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O37" s="4" t="s">
-        <v>164</v>
+        <v>127</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C38" s="3">
         <v>22</v>
@@ -2395,31 +2275,31 @@
         <v>1</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="L38" s="3">
         <v>60</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O38" s="3"/>
       <c r="P38" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="39" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C39" s="3">
         <v>259</v>
@@ -2428,31 +2308,31 @@
         <v>1</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="L39" s="3">
         <v>54</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O39" s="3"/>
       <c r="P39" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="40" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C40" s="3">
         <v>127</v>
@@ -2461,31 +2341,31 @@
         <v>1</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="L40" s="3">
         <v>54</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O40" s="3"/>
       <c r="P40" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="41" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C41" s="3">
         <v>113.2</v>
@@ -2494,33 +2374,33 @@
         <v>1</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="L41" s="3">
         <v>35</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>180</v>
+        <v>142</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="42" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C42" s="3">
         <v>115</v>
@@ -2529,37 +2409,37 @@
         <v>1</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
       <c r="L42" s="3">
         <v>65</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O42" s="3"/>
       <c r="P42" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="43" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C43" s="3">
-        <v>64.900000000000006</v>
+        <v>138.6</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G43" s="3">
         <v>3.7699999999999997E-2</v>
@@ -2571,29 +2451,31 @@
         <v>0.34949999999999998</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>168</v>
+        <v>131</v>
       </c>
       <c r="L43" s="3">
         <v>31</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O43" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="O43" s="3" t="s">
+        <v>164</v>
+      </c>
       <c r="P43" s="3" t="s">
-        <v>96</v>
+        <v>169</v>
       </c>
       <c r="Q43" s="3"/>
     </row>
-    <row r="44" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C44">
         <v>187</v>
@@ -2602,31 +2484,31 @@
         <v>1</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="L44" s="3">
         <v>73</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O44" s="3"/>
       <c r="P44" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="45" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C45" s="3">
         <v>22.2</v>
@@ -2635,78 +2517,80 @@
         <v>1</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="L45" s="3">
         <v>36</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O45" s="3" t="s">
-        <v>181</v>
+        <v>143</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q45" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="46" spans="1:18" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C46" s="6">
-        <f>424.5/3.32</f>
-        <v>127.86144578313254</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="6">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C46" s="3">
+        <v>127.9</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="3">
         <v>0.83199999999999996</v>
       </c>
-      <c r="F46" s="6">
+      <c r="F46" s="3">
         <v>28.478999999999999</v>
       </c>
-      <c r="K46" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="L46" s="6">
+      <c r="K46" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L46" s="3">
         <v>53</v>
       </c>
-      <c r="M46" s="6" t="s">
-        <v>92</v>
+      <c r="M46" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="N46" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O46" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="P46" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="47" spans="1:18" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+      <c r="O46" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q46" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C47" s="4">
         <v>2272.5</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E47" s="4">
         <v>0.35930000000000001</v>
@@ -2715,39 +2599,39 @@
         <v>12.45</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="L47" s="4">
         <v>53</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O47" s="4" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="P47" s="4" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="Q47" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="48" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C48" s="3">
         <v>322</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G48" s="3">
         <v>9.3649999999999997E-2</v>
@@ -2759,34 +2643,34 @@
         <v>0.50360000000000005</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="L48" s="3">
         <v>32</v>
       </c>
       <c r="M48" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N48" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O48" s="4" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="P48" s="3" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="Q48" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="R48" s="4"/>
     </row>
-    <row r="49" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C49" s="3">
         <v>70</v>
@@ -2795,31 +2679,31 @@
         <v>1</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="L49" s="4">
         <v>66</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N49" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O49" s="3"/>
       <c r="P49" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q49" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="50" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C50" s="3">
         <v>13</v>
@@ -2828,41 +2712,41 @@
         <v>1</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="L50" s="4">
         <v>50</v>
       </c>
       <c r="M50" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N50" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O50" s="3"/>
       <c r="P50" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q50" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="51" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C51" s="4">
         <v>495</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
-      <c r="G51" s="12">
+      <c r="G51" s="9">
         <v>1.9699999999999999E-2</v>
       </c>
       <c r="H51" s="4">
@@ -2873,31 +2757,31 @@
       </c>
       <c r="J51" s="4"/>
       <c r="K51" s="4" t="s">
-        <v>196</v>
+        <v>157</v>
       </c>
       <c r="L51" s="4">
         <v>64</v>
       </c>
       <c r="M51" s="5" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N51" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O51" s="4"/>
       <c r="P51" s="4" t="s">
-        <v>197</v>
+        <v>158</v>
       </c>
       <c r="Q51" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="52" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C52">
         <v>54</v>
@@ -2906,30 +2790,30 @@
         <v>1</v>
       </c>
       <c r="K52" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="L52" s="4">
         <v>54</v>
       </c>
-      <c r="M52" s="10" t="s">
-        <v>162</v>
+      <c r="M52" s="8" t="s">
+        <v>125</v>
       </c>
       <c r="N52" s="3" t="s">
-        <v>198</v>
+        <v>159</v>
       </c>
       <c r="P52" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q52" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C53" s="3">
         <v>53.6</v>
@@ -2938,28 +2822,30 @@
         <v>1</v>
       </c>
       <c r="K53" s="3" t="s">
-        <v>182</v>
+        <v>144</v>
       </c>
       <c r="L53" s="4">
         <v>69</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="P53" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q53" s="4"/>
-    </row>
-    <row r="54" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+      <c r="Q53" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>183</v>
+        <v>145</v>
       </c>
       <c r="C54">
         <v>55.7</v>
@@ -2968,33 +2854,31 @@
         <v>1</v>
       </c>
       <c r="K54" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="L54" s="3">
         <v>44</v>
       </c>
       <c r="M54" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N54" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O54" s="3" t="s">
-        <v>183</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="O54" s="3"/>
       <c r="P54" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q54" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C55" s="3">
         <v>91.6</v>
@@ -3003,31 +2887,31 @@
         <v>1</v>
       </c>
       <c r="K55" s="3" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="L55" s="3">
         <v>46</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N55" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O55" s="3"/>
       <c r="P55" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q55" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C56" s="3">
         <v>154.30000000000001</v>
@@ -3036,31 +2920,31 @@
         <v>1</v>
       </c>
       <c r="K56" s="3" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="L56" s="3">
         <v>39</v>
       </c>
       <c r="M56" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N56" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O56" s="3"/>
       <c r="P56" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q56" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="57" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>183</v>
+        <v>145</v>
       </c>
       <c r="C57" s="3">
         <v>22.4</v>
@@ -3069,33 +2953,31 @@
         <v>1</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>170</v>
+        <v>133</v>
       </c>
       <c r="L57" s="3">
         <v>20</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N57" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="O57" s="3" t="s">
-        <v>183</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="O57" s="3"/>
       <c r="P57" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q57" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="58" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C58" s="3">
         <v>46.6</v>
@@ -3104,33 +2986,33 @@
         <v>1</v>
       </c>
       <c r="K58" s="3" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="L58" s="3">
         <v>64</v>
       </c>
-      <c r="M58" s="10" t="s">
-        <v>162</v>
+      <c r="M58" s="8" t="s">
+        <v>125</v>
       </c>
       <c r="N58" s="3" t="s">
-        <v>199</v>
+        <v>160</v>
       </c>
       <c r="O58" s="3" t="s">
-        <v>200</v>
+        <v>161</v>
       </c>
       <c r="P58" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q58" s="3" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="59" spans="1:17" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C59" s="3">
         <v>149.9</v>
@@ -3139,33 +3021,33 @@
         <v>1</v>
       </c>
       <c r="K59" s="3" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="L59" s="3">
         <v>64</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N59" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O59" s="3" t="s">
-        <v>201</v>
+        <v>162</v>
       </c>
       <c r="P59" s="3" t="s">
-        <v>197</v>
+        <v>158</v>
       </c>
       <c r="Q59" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="60" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C60" s="3">
         <v>16.8</v>
@@ -3174,31 +3056,31 @@
         <v>1</v>
       </c>
       <c r="K60" s="3" t="s">
-        <v>166</v>
+        <v>129</v>
       </c>
       <c r="L60" s="3">
         <v>44</v>
       </c>
       <c r="M60" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N60" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O60" s="3"/>
       <c r="P60" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q60" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="61" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="C61" s="3">
         <v>6.71</v>
@@ -3207,23 +3089,23 @@
         <v>1</v>
       </c>
       <c r="K61" s="3" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="L61" s="3">
         <v>37</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N61" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O61" s="3"/>
       <c r="P61" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="Q61" s="3" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -3238,222 +3120,4 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EAD96ED-6947-4032-A468-AE450047F46C}">
-  <dimension ref="A1:B26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>126</v>
-      </c>
-      <c r="B9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B15" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>73</v>
-      </c>
-      <c r="B21" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>65</v>
-      </c>
-      <c r="B23" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>138</v>
-      </c>
-      <c r="B24" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>139</v>
-      </c>
-      <c r="B25" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" t="s">
-        <v>141</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>